<commit_message>
Add send-ready outreach workspace
</commit_message>
<xml_diff>
--- a/zh/outreach-tracker.xlsx
+++ b/zh/outreach-tracker.xlsx
@@ -4897,7 +4897,7 @@
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>first-five-micro-audits.md#1-virling</t>
+          <t>outreach/send-ready.html#virling</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
@@ -4905,10 +4905,6 @@
           <t>待发送确认</t>
         </is>
       </c>
-      <c r="H501" t="inlineStr"/>
-      <c r="I501" t="inlineStr"/>
-      <c r="J501" t="inlineStr"/>
-      <c r="K501" t="inlineStr"/>
       <c r="L501" t="inlineStr">
         <is>
           <t>待发送确认</t>
@@ -4953,7 +4949,7 @@
       </c>
       <c r="F502" t="inlineStr">
         <is>
-          <t>first-five-micro-audits.md#2-papertrail</t>
+          <t>outreach/send-ready.html#papertrail</t>
         </is>
       </c>
       <c r="G502" t="inlineStr">
@@ -4961,10 +4957,6 @@
           <t>待发送确认</t>
         </is>
       </c>
-      <c r="H502" t="inlineStr"/>
-      <c r="I502" t="inlineStr"/>
-      <c r="J502" t="inlineStr"/>
-      <c r="K502" t="inlineStr"/>
       <c r="L502" t="inlineStr">
         <is>
           <t>待发送确认</t>
@@ -5009,7 +5001,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>first-five-micro-audits.md#3-menivor</t>
+          <t>outreach/send-ready.html#menivor</t>
         </is>
       </c>
       <c r="G503" t="inlineStr">
@@ -5017,10 +5009,6 @@
           <t>待发送确认</t>
         </is>
       </c>
-      <c r="H503" t="inlineStr"/>
-      <c r="I503" t="inlineStr"/>
-      <c r="J503" t="inlineStr"/>
-      <c r="K503" t="inlineStr"/>
       <c r="L503" t="inlineStr">
         <is>
           <t>待发送确认</t>
@@ -5065,7 +5053,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>first-five-micro-audits.md#4-megaphone</t>
+          <t>outreach/send-ready.html#megaphone</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -5073,10 +5061,6 @@
           <t>待发送确认</t>
         </is>
       </c>
-      <c r="H504" t="inlineStr"/>
-      <c r="I504" t="inlineStr"/>
-      <c r="J504" t="inlineStr"/>
-      <c r="K504" t="inlineStr"/>
       <c r="L504" t="inlineStr">
         <is>
           <t>待发送确认</t>
@@ -5121,7 +5105,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>first-five-micro-audits.md#5-worksitem</t>
+          <t>outreach/send-ready.html#worksitem</t>
         </is>
       </c>
       <c r="G505" t="inlineStr">
@@ -5129,10 +5113,6 @@
           <t>待发送确认</t>
         </is>
       </c>
-      <c r="H505" t="inlineStr"/>
-      <c r="I505" t="inlineStr"/>
-      <c r="J505" t="inlineStr"/>
-      <c r="K505" t="inlineStr"/>
       <c r="L505" t="inlineStr">
         <is>
           <t>待发送确认</t>

</xml_diff>